<commit_message>
docs(reports): v0.2.1~v0.2.3 commit 改 DRAFT + note 加前置/依赖
- v0.2.1 commit: 33cfd0f → DRAFT；note: 未开始；用户在 oa.dingtalk.com 建模板
- v0.2.2 commit: 33cfd0f → DRAFT；note: 前置条件 DBA 需自备域名（公网已备案），
  不能用 trycloudflare 临时域名，callback URL 走域名+HTTPS
- v0.2.3 commit: 33cfd0f → DRAFT；note: 依赖 v0.2.1 模板 + v0.2.2 tunnel 都完成后
  才能做（callback 不通就没法对账）
</commit_message>
<xml_diff>
--- a/docs/reports/2026-08-06_功能开发计划_v3.xlsx
+++ b/docs/reports/2026-08-06_功能开发计划_v3.xlsx
@@ -2467,7 +2467,7 @@
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>33cfd0f</t>
+          <t>DRAFT</t>
         </is>
       </c>
       <c r="G33" s="12" t="inlineStr">
@@ -2485,7 +2485,11 @@
           <t>0.5</t>
         </is>
       </c>
-      <c r="J33" s="9" t="inlineStr"/>
+      <c r="J33" s="9" t="inlineStr">
+        <is>
+          <t>未开始；用户在 oa.dingtalk.com 建模板</t>
+        </is>
+      </c>
       <c r="K33" s="10" t="inlineStr"/>
     </row>
     <row r="34" ht="24" customHeight="1">
@@ -2516,7 +2520,7 @@
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>33cfd0f</t>
+          <t>DRAFT</t>
         </is>
       </c>
       <c r="G34" s="12" t="inlineStr">
@@ -2534,7 +2538,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="J34" s="9" t="inlineStr"/>
+      <c r="J34" s="9" t="inlineStr">
+        <is>
+          <t>前置条件：DBA 需自备域名（公网已备案），不能用 trycloudflare 临时域名；callback URL 走域名 + HTTPS</t>
+        </is>
+      </c>
       <c r="K34" s="10" t="inlineStr"/>
     </row>
     <row r="35" ht="24" customHeight="1">
@@ -2565,7 +2573,7 @@
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>33cfd0f</t>
+          <t>DRAFT</t>
         </is>
       </c>
       <c r="G35" s="12" t="inlineStr">
@@ -2583,7 +2591,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="J35" s="9" t="inlineStr"/>
+      <c r="J35" s="9" t="inlineStr">
+        <is>
+          <t>依赖：v0.2.1 模板 + v0.2.2 tunnel 都完成后才能做（callback 不通就没法对账）</t>
+        </is>
+      </c>
       <c r="K35" s="10" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(reports): v0.4.0 标已发布 + v0.4.5-alpha 加 6 行规划
- v0.4.0 列压缩：状态 已发布 + commit 33cfd0f（清 row 32 重复行）
- v0.4.5-alpha 碎片回收 6 行规划（model/service/view/admin/queue/演练）
  - 全部 DRAFT + 待办，等 v0.4.5-alpha 实现时替换

设计拍板（2026-08-06）：
- 复用 ext_ddl_ghost_task + task_type 字段
- DBA 手动 + 一键批量默认开，归档联动 + cron 默认关
- v0.4.1 归档 和 v0.4.5 重建 是两个独立 task
- 同表冲突 → 排队（先归档后重建）

CHANGELOG: docs/changelogs/2026-08-06_v045-planning.md
</commit_message>
<xml_diff>
--- a/docs/reports/2026-08-06_功能开发计划_v3.xlsx
+++ b/docs/reports/2026-08-06_功能开发计划_v3.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="49">
+  <fonts count="56">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -361,8 +361,47 @@
       <color rgb="001F5B96"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0014171E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="003A4256"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="009C5700"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002F6F5E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <i val="1"/>
+      <color rgb="009C5700"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="50">
+  <fills count="56">
     <fill>
       <patternFill/>
     </fill>
@@ -648,6 +687,36 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EAF1F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F0ED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBF1E4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -934,7 +1003,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1080,6 +1149,48 @@
     </xf>
     <xf numFmtId="0" fontId="48" fillId="49" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="50" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="50" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="51" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="52" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="43" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="49" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="53" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="54" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="55" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1493,7 +1604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3133,91 +3244,103 @@
           <t>v0.4.0 列压缩</t>
         </is>
       </c>
-      <c r="C31" s="25" t="inlineStr">
+      <c r="C31" s="54" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="D31" s="36" t="inlineStr">
+      <c r="D31" s="55" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E31" s="56" t="inlineStr">
+        <is>
+          <t>已发布</t>
+        </is>
+      </c>
+      <c r="F31" s="57" t="inlineStr">
+        <is>
+          <t>33cfd0f</t>
+        </is>
+      </c>
+      <c r="G31" s="58" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H31" s="59" t="inlineStr">
+        <is>
+          <t>mavis</t>
+        </is>
+      </c>
+      <c r="I31" s="53" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="J31" s="60" t="inlineStr">
+        <is>
+          <t>Excel 列压缩到 11 列；DROP COLUMN + ADD COLUMN 改写为单行 ALTER 链</t>
+        </is>
+      </c>
+      <c r="K31" s="61" t="inlineStr">
+        <is>
+          <t>【场景】v0.3.0 之前 DROP/ADD 拆成两条工单，134 dev 演练 1 张表要走 2 次 gh-ost。【使用】工单页面检测到 DROP+ADD 同表同提交 → 合并成 `ALTER TABLE x DROP col_a, ADD col_b` 单条 → 1 次 gh-ost 完成。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="48" customHeight="1">
+      <c r="A32" s="33" t="inlineStr">
+        <is>
+          <t>钉钉 OA 集成</t>
+        </is>
+      </c>
+      <c r="B32" s="25" t="inlineStr">
+        <is>
+          <t>v0.2.1 钉钉 OA 模板（process_code）</t>
+        </is>
+      </c>
+      <c r="C32" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D32" s="36" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="E31" s="34" t="inlineStr">
+      <c r="E32" s="34" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="F31" s="28" t="inlineStr">
-        <is>
-          <t>2c5a0b7</t>
-        </is>
-      </c>
-      <c r="G31" s="34" t="inlineStr">
+      <c r="F32" s="28" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="G32" s="34" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H31" s="29" t="inlineStr">
+      <c r="H32" s="29" t="inlineStr">
         <is>
           <t>马克群</t>
         </is>
       </c>
-      <c r="I31" s="53" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="J31" s="42" t="inlineStr"/>
-      <c r="K31" s="50" t="inlineStr"/>
-    </row>
-    <row r="32" ht="48" customHeight="1">
-      <c r="A32" s="35" t="inlineStr">
-        <is>
-          <t>gh-ost 无锁 DDL</t>
-        </is>
-      </c>
-      <c r="B32" s="25" t="inlineStr">
-        <is>
-          <t>v0.4.0 列压缩</t>
-        </is>
-      </c>
-      <c r="C32" s="25" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="D32" s="36" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="E32" s="34" t="inlineStr">
-        <is>
-          <t>待办</t>
-        </is>
-      </c>
-      <c r="F32" s="28" t="inlineStr">
-        <is>
-          <t>8d78389</t>
-        </is>
-      </c>
-      <c r="G32" s="34" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="H32" s="29" t="inlineStr">
-        <is>
-          <t>马克群</t>
-        </is>
-      </c>
       <c r="I32" s="53" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="J32" s="42" t="inlineStr"/>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="J32" s="43" t="inlineStr">
+        <is>
+          <t>未开始；用户在 oa.dingtalk.com 建模板</t>
+        </is>
+      </c>
       <c r="K32" s="50" t="inlineStr"/>
     </row>
     <row r="33" ht="24" customHeight="1">
@@ -3228,7 +3351,7 @@
       </c>
       <c r="B33" s="25" t="inlineStr">
         <is>
-          <t>v0.2.1 钉钉 OA 模板（process_code）</t>
+          <t>v0.2.2 Tunnel + 回调加密（cloudflared）</t>
         </is>
       </c>
       <c r="C33" s="25" t="inlineStr">
@@ -3263,12 +3386,12 @@
       </c>
       <c r="I33" s="53" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J33" s="43" t="inlineStr">
         <is>
-          <t>未开始；用户在 oa.dingtalk.com 建模板</t>
+          <t>前置条件：DBA 需自备域名（公网已备案），不能用 trycloudflare 临时域名；callback URL 走域名 + HTTPS</t>
         </is>
       </c>
       <c r="K33" s="50" t="inlineStr"/>
@@ -3281,7 +3404,7 @@
       </c>
       <c r="B34" s="25" t="inlineStr">
         <is>
-          <t>v0.2.2 Tunnel + 回调加密（cloudflared）</t>
+          <t>v0.2.3 对账 cron + runbook</t>
         </is>
       </c>
       <c r="C34" s="25" t="inlineStr">
@@ -3321,63 +3444,340 @@
       </c>
       <c r="J34" s="43" t="inlineStr">
         <is>
-          <t>前置条件：DBA 需自备域名（公网已备案），不能用 trycloudflare 临时域名；callback URL 走域名 + HTTPS</t>
+          <t>依赖：v0.2.1 模板 + v0.2.2 tunnel 都完成后才能做（callback 不通就没法对账）</t>
         </is>
       </c>
       <c r="K34" s="50" t="inlineStr"/>
     </row>
-    <row r="35" ht="24" customHeight="1">
-      <c r="A35" s="33" t="inlineStr">
-        <is>
-          <t>钉钉 OA 集成</t>
-        </is>
-      </c>
-      <c r="B35" s="25" t="inlineStr">
-        <is>
-          <t>v0.2.3 对账 cron + runbook</t>
-        </is>
-      </c>
-      <c r="C35" s="25" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="D35" s="36" t="inlineStr">
+    <row r="35" ht="56" customHeight="1">
+      <c r="A35" s="62" t="inlineStr">
+        <is>
+          <t>gh-ost 无锁 DDL</t>
+        </is>
+      </c>
+      <c r="B35" s="63" t="inlineStr">
+        <is>
+          <t>v0.4.5-alpha：model 改造（task_type + target_table + 拆 OneToOne）</t>
+        </is>
+      </c>
+      <c r="C35" s="64" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D35" s="65" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="E35" s="34" t="inlineStr">
+      <c r="E35" s="58" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="F35" s="28" t="inlineStr">
+      <c r="F35" s="66" t="inlineStr">
         <is>
           <t>DRAFT</t>
         </is>
       </c>
-      <c r="G35" s="34" t="inlineStr">
+      <c r="G35" s="58" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H35" s="29" t="inlineStr">
-        <is>
-          <t>马克群</t>
-        </is>
-      </c>
-      <c r="I35" s="53" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="J35" s="43" t="inlineStr">
-        <is>
-          <t>依赖：v0.2.1 模板 + v0.2.2 tunnel 都完成后才能做（callback 不通就没法对账）</t>
-        </is>
-      </c>
-      <c r="K35" s="50" t="inlineStr"/>
+      <c r="H35" s="59" t="inlineStr">
+        <is>
+          <t>mavis</t>
+        </is>
+      </c>
+      <c r="I35" s="53" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J35" s="67" t="inlineStr">
+        <is>
+          <t>拆 OneToOne 为 ForeignKey(null)；task_type 区分 ghost/rebuild；Meta.unique_together 约束</t>
+        </is>
+      </c>
+      <c r="K35" s="50" t="inlineStr">
+        <is>
+          <t>【场景】ghost 是工单级（OneToOne SqlWorkflow），rebuild 是表级（DBA 手动选表）。【使用】新增字段 `task_type`/`target_table`/`related_task_id`；rebuild 时 workflow=NULL，target_table 存 `db.table`。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="56" customHeight="1">
+      <c r="A36" s="62" t="inlineStr">
+        <is>
+          <t>gh-ost 无锁 DDL</t>
+        </is>
+      </c>
+      <c r="B36" s="63" t="inlineStr">
+        <is>
+          <t>v0.4.5-alpha：rebuild service（services/rebuild.py）</t>
+        </is>
+      </c>
+      <c r="C36" s="64" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D36" s="65" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E36" s="58" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="F36" s="66" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="G36" s="56" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H36" s="59" t="inlineStr">
+        <is>
+          <t>mavis</t>
+        </is>
+      </c>
+      <c r="I36" s="53" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J36" s="67" t="inlineStr">
+        <is>
+          <t>复用 runner.py，差别只在 --alter 改 COMMENT 空 alter 触发重建</t>
+        </is>
+      </c>
+      <c r="K36" s="50" t="inlineStr">
+        <is>
+          <t>【场景】大表碎片率高，OPTIMIZE TABLE 锁表；pt-osc 装新环境成本高。【使用】gh-ost 跑 `ALTER TABLE x COMMENT 'archery-auto-rebuild-YYYYMMDD'`，结构不变触发表重建，几秒锁表完成。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="56" customHeight="1">
+      <c r="A37" s="62" t="inlineStr">
+        <is>
+          <t>gh-ost 无锁 DDL</t>
+        </is>
+      </c>
+      <c r="B37" s="63" t="inlineStr">
+        <is>
+          <t>v0.4.5-alpha：视图 + 路由（rebuild/list 端点）</t>
+        </is>
+      </c>
+      <c r="C37" s="64" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D37" s="65" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E37" s="58" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="F37" s="66" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="G37" s="58" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H37" s="59" t="inlineStr">
+        <is>
+          <t>mavis</t>
+        </is>
+      </c>
+      <c r="I37" s="53" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J37" s="67" t="inlineStr">
+        <is>
+          <t>新增 POST /gh_ost/rebuild/&lt;table_id&gt;/ + GET /gh_ost/rebuild/list/</t>
+        </is>
+      </c>
+      <c r="K37" s="50" t="inlineStr">
+        <is>
+          <t>【场景】DBA 选 instance + 表 → 一键触发 rebuild。【使用】DBA 在 admin 表列表点 "重建" → 写 task（task_type=rebuild, workflow=NULL）→ 启动 gh-ost → 进度面板 polling 3s。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="56" customHeight="1">
+      <c r="A38" s="62" t="inlineStr">
+        <is>
+          <t>gh-ost 无锁 DDL</t>
+        </is>
+      </c>
+      <c r="B38" s="63" t="inlineStr">
+        <is>
+          <t>v0.4.5-alpha：admin + UI（list_filter + 批量 action）</t>
+        </is>
+      </c>
+      <c r="C38" s="64" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D38" s="65" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E38" s="58" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="F38" s="66" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="G38" s="58" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H38" s="59" t="inlineStr">
+        <is>
+          <t>mavis</t>
+        </is>
+      </c>
+      <c r="I38" s="53" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J38" s="67" t="inlineStr">
+        <is>
+          <t>admin list_filter 加 task_type；admin action 加 "批量重建"；progress.html 适配 rebuild 无工单场景</t>
+        </is>
+      </c>
+      <c r="K38" s="50" t="inlineStr">
+        <is>
+          <t>【场景】DBA 看到一堆要重建的表，挨个点太慢。【使用】admin 勾选 N 张表 → action 选 "批量重建" → 一次触发 N 个 rebuild task（按表排队，同表只跑 1 个）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="56" customHeight="1">
+      <c r="A39" s="62" t="inlineStr">
+        <is>
+          <t>gh-ost 无锁 DDL</t>
+        </is>
+      </c>
+      <c r="B39" s="63" t="inlineStr">
+        <is>
+          <t>v0.4.5-alpha：排队 + 关联归档（services/queue.py）</t>
+        </is>
+      </c>
+      <c r="C39" s="64" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D39" s="65" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E39" s="58" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="F39" s="66" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="G39" s="58" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H39" s="59" t="inlineStr">
+        <is>
+          <t>mavis</t>
+        </is>
+      </c>
+      <c r="I39" s="53" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J39" s="67" t="inlineStr">
+        <is>
+          <t>同表冲突排队（FIFO）；归档联动 auto_link_archive opt-in 开关</t>
+        </is>
+      </c>
+      <c r="K39" s="50" t="inlineStr">
+        <is>
+          <t>【场景】DBA 同时点 "归档 + 回收"，同表 2 个 task 撞车。【使用】rebuild 检测到同表有归档 task running → 排队等前面完成 → 归档完自动启动 rebuild。归档联动默认关，要开显式勾 "归档完自动回收"。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="56" customHeight="1">
+      <c r="A40" s="62" t="inlineStr">
+        <is>
+          <t>gh-ost 无锁 DDL</t>
+        </is>
+      </c>
+      <c r="B40" s="63" t="inlineStr">
+        <is>
+          <t>v0.4.5-alpha：134 dev 演练（accesscard_black_detail 造碎片 → 重建）</t>
+        </is>
+      </c>
+      <c r="C40" s="64" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D40" s="65" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E40" s="58" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="F40" s="66" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="G40" s="58" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H40" s="59" t="inlineStr">
+        <is>
+          <t>mavis</t>
+        </is>
+      </c>
+      <c r="I40" s="53" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J40" s="67" t="inlineStr">
+        <is>
+          <t>删 50% 数据造碎片 → 跑 rebuild → 前后对比 INFORMATION_SCHEMA.TABLES.DATA_FREE</t>
+        </is>
+      </c>
+      <c r="K40" s="50" t="inlineStr">
+        <is>
+          <t>【场景】真实业务表测碎片回收效果。【使用】DBA 在 134 dev dev 库演练大表 accesscard_black_detail 上删一半行 → 点重建 → 观察 gh-ost 进度 → 验证 DATA_FREE 下降。重复 1 表 N 次验证限频 1 次/天/表。</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(reports): v0.4.0 归档专题 全套规划入表（v0.4.1~v0.4.3 + v0.4.5）
新增 7 行规划（row 32-38）：

- v0.4.1 现有归档补强（3 行）：
  * ArchiveConfig 加进度字段（last_archive_status + progress_pct）
  * 归档详情页增强（archive_detail.html 进度条 + 历史日志表格）
  * 归档完成钉钉通知

- v0.4.2 归档→重建联动（2 行）：
  * ArchiveConfig 加 auto_rebuild_after_archive 字段
  * 134 dev 演练归档→自动回收

- v0.4.3 归档审计页（2 行）：
  * ArchiveLog 前端表格化
  * 归档成功率统计 dashboard

设计拍板（2026-08-06）：
- v0.4.1~v0.4.3 全部基于现有 ArchiveConfig / ArchiveLog / archiver.py 补强
- v0.4.2 联动 v0.4.5 走 auto_rebuild_after_archive Boolean 字段（每条归档独立勾选）
- v0.4.5 碎片回收 6 行（model/service/view/admin/queue/演练）保持 DRAFT

修 col 1 错位：原 v0.2.x 行被下移后 col1 丢，统一 unmerge 错位 merges + 重写 col 1

CHANGELOG: docs/changelogs/2026-08-06_v040-archive-planning.md
</commit_message>
<xml_diff>
--- a/docs/reports/2026-08-06_功能开发计划_v3.xlsx
+++ b/docs/reports/2026-08-06_功能开发计划_v3.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="56">
+  <fonts count="55">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -159,22 +159,51 @@
       <name val="Calibri"/>
       <charset val="134"/>
       <b val="1"/>
+      <color rgb="FF1F3A5F"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color rgb="FF9C2A00"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color rgb="FF3A2E1F"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
       <color rgb="FF595959"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="FFC00000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color rgb="FF14171E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
       <charset val="134"/>
       <i val="1"/>
       <color rgb="FF9C5700"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="宋体"/>
@@ -322,38 +351,37 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00595959"/>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="0014171E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="003A2E1F"/>
-      <sz val="9.5"/>
+      <color rgb="009C5700"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <i val="1"/>
+      <color rgb="009C5700"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="009C2A00"/>
-      <sz val="9.5"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="0014171E"/>
-      <sz val="9.5"/>
+      <color rgb="00006100"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <i val="1"/>
-      <color rgb="00C00000"/>
+      <color rgb="002F6F5E"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001F3A5F"/>
-      <sz val="9.5"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -363,45 +391,16 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="0014171E"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00006100"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Consolas"/>
-      <color rgb="003A4256"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="009C5700"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="002F6F5E"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Consolas"/>
-      <i val="1"/>
-      <color rgb="009C5700"/>
-      <sz val="9"/>
+      <sz val="9.5"/>
     </font>
   </fonts>
-  <fills count="56">
+  <fills count="54">
     <fill>
       <patternFill/>
     </fill>
@@ -464,12 +463,48 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFE5F0FA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE5CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF8DC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFD9D9D9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFE5E5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD580"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF4D6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -494,24 +529,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -656,12 +673,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF8DC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFD580"/>
+        <fgColor rgb="00FBF1E4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F0ED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF1F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -669,58 +711,8 @@
         <fgColor rgb="00FAF8F0"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFE5E5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E5F0FA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFE5CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EAF1F8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8F0ED"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FBF1E4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF4D6"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="11">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -738,6 +730,43 @@
       <top style="thin">
         <color rgb="FFBFBFBF"/>
       </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
       <bottom style="thin">
         <color rgb="FFBFBFBF"/>
       </bottom>
@@ -843,6 +872,15 @@
     </border>
     <border>
       <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="00BFBFBF"/>
       </left>
       <right style="thin">
@@ -855,155 +893,188 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="22" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="22" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="22" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="22" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="22" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="3" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="3" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="4" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="13" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="14" borderId="6" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="14" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="15" borderId="7" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="8" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="9" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="16" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="17" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="18" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="19" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="20" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="21" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="22" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="23" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="24" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="25" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="26" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="27" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="28" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="29" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="30" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="31" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="32" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="33" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="34" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="35" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="36" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="37" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="38" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="39" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="40" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="41" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="42" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="19" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="20" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="20" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="21" borderId="10" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="11" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="12" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="5" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="6" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="34" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="35" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="36" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="37" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="38" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="39" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="40" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="41" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="42" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="43" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="44" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="45" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1087,6 +1158,9 @@
     <xf numFmtId="0" fontId="19" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1096,10 +1170,16 @@
     <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1108,17 +1188,88 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="43" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="44" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="46" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="47" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="48" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="49" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="50" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="51" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="52" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="53" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1135,61 +1286,7 @@
     <xf numFmtId="164" fontId="14" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="46" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="45" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="47" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="48" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="49" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="50" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="50" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="52" fillId="51" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="53" fillId="52" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="43" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="49" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="53" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="54" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="55" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="51" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1604,7 +1701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1721,17 +1818,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I2" s="53" t="inlineStr">
+      <c r="I2" s="30" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="J2" s="41" t="inlineStr">
+      <c r="J2" s="31" t="inlineStr">
         <is>
           <t>基线版本，3 套环境脚手架</t>
         </is>
       </c>
-      <c r="K2" s="50" t="inlineStr">
+      <c r="K2" s="32" t="inlineStr">
         <is>
           <t>【场景】公司 DBA 团队需要 SQL 审核 + 工单流平台；【使用】部署后默认进入 Archery 主界面，业务开发走标准 SQL 上线流程。</t>
         </is>
@@ -1774,17 +1871,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I3" s="53" t="inlineStr">
+      <c r="I3" s="30" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="J3" s="41" t="inlineStr">
+      <c r="J3" s="31" t="inlineStr">
         <is>
           <t>dev=9003 / prod=9123，裸机 systemd</t>
         </is>
       </c>
-      <c r="K3" s="51" t="inlineStr">
+      <c r="K3" s="33" t="inlineStr">
         <is>
           <t>【场景】3 套环境隔离，代码不直接动生产；【使用】每套独立 .env + systemd unit，promote_110.sh 跨环境发布。</t>
         </is>
@@ -1827,17 +1924,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I4" s="53" t="inlineStr">
+      <c r="I4" s="30" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="J4" s="41" t="inlineStr">
+      <c r="J4" s="31" t="inlineStr">
         <is>
           <t>systemd 化、qcluster 配置、ARCHERY_LOG_LEVEL</t>
         </is>
       </c>
-      <c r="K4" s="51" t="inlineStr">
+      <c r="K4" s="33" t="inlineStr">
         <is>
           <t>【场景】dev 从手工启服务到稳定 systemd；【使用】systemctl start archery-prod-gunicorn / archery-prod-qcluster，journalctl -u 看日志。</t>
         </is>
@@ -1880,17 +1977,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I5" s="53" t="inlineStr">
+      <c r="I5" s="30" t="inlineStr">
         <is>
           <t>0.1</t>
         </is>
       </c>
-      <c r="J5" s="41" t="inlineStr">
+      <c r="J5" s="31" t="inlineStr">
         <is>
           <t>134=DEV / 110=PROD</t>
         </is>
       </c>
-      <c r="K5" s="51" t="inlineStr">
+      <c r="K5" s="33" t="inlineStr">
         <is>
           <t>【场景】防止误操作生产；【使用】dev 验证通过才推 prod，110 prod 仅手动 ssh 介入。</t>
         </is>
@@ -1933,24 +2030,24 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I6" s="53" t="inlineStr">
+      <c r="I6" s="30" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="J6" s="41" t="inlineStr">
+      <c r="J6" s="31" t="inlineStr">
         <is>
           <t>5 phase 发布脚本</t>
         </is>
       </c>
-      <c r="K6" s="51" t="inlineStr">
+      <c r="K6" s="33" t="inlineStr">
         <is>
           <t>【场景】134 dev 验证完要一键推到 110 prod；【使用】在 134 上跑 ./scripts/promote_110.sh &lt;commit-hash&gt;，自动 backup + fetch + adapt + deploy。</t>
         </is>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="33" t="inlineStr">
+      <c r="A7" s="34" t="inlineStr">
         <is>
           <t>钉钉 OA 集成</t>
         </is>
@@ -1990,17 +2087,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I7" s="53" t="inlineStr">
+      <c r="I7" s="30" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="J7" s="41" t="inlineStr">
+      <c r="J7" s="31" t="inlineStr">
         <is>
           <t>audit_driver 可扩展</t>
         </is>
       </c>
-      <c r="K7" s="51" t="inlineStr">
+      <c r="K7" s="33" t="inlineStr">
         <is>
           <t>【场景】未来想接入企业微信 OA / 飞书审批不用改核心；【使用】DRIVER_REGISTRY 注册新 driver，admin 配置 flow.audit_driver 选新值即可。</t>
         </is>
@@ -2043,17 +2140,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I8" s="53" t="inlineStr">
+      <c r="I8" s="30" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="J8" s="41" t="inlineStr">
+      <c r="J8" s="31" t="inlineStr">
         <is>
           <t>SQL 类型∧核心表∧行数</t>
         </is>
       </c>
-      <c r="K8" s="50" t="inlineStr">
+      <c r="K8" s="32" t="inlineStr">
         <is>
           <t>【场景】不同 SQL 类型 + 不同业务表 + 不同行数走不同审批；【使用】admin 维护 ext_approval_policy 多条规则，按 priority 倒序匹配。</t>
         </is>
@@ -2096,17 +2193,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I9" s="53" t="inlineStr">
+      <c r="I9" s="30" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="J9" s="41" t="inlineStr">
+      <c r="J9" s="31" t="inlineStr">
         <is>
           <t>select_for_update + 验签</t>
         </is>
       </c>
-      <c r="K9" s="51" t="inlineStr">
+      <c r="K9" s="33" t="inlineStr">
         <is>
           <t>【场景】钉钉侧审批结果自动回写到 Archery 状态；【使用】钉钉推送 → /dingtalk/oa/callback → 自动推进工单 + 写 WorkflowAuditDetail。</t>
         </is>
@@ -2149,17 +2246,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I10" s="53" t="inlineStr">
+      <c r="I10" s="30" t="inlineStr">
         <is>
           <t>0.3</t>
         </is>
       </c>
-      <c r="J10" s="41" t="inlineStr">
+      <c r="J10" s="31" t="inlineStr">
         <is>
           <t>workflow_id=4 真跑通</t>
         </is>
       </c>
-      <c r="K10" s="50" t="inlineStr">
+      <c r="K10" s="32" t="inlineStr">
         <is>
           <t>【场景】审批人变更时主动通知；【使用】dingtalk_oa driver 自动调钉钉 Open API 推 1对1 消息，业务方无需手动。</t>
         </is>
@@ -2192,7 +2289,7 @@
           <t>c9236a0</t>
         </is>
       </c>
-      <c r="G11" s="34" t="inlineStr">
+      <c r="G11" s="35" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -2202,17 +2299,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I11" s="53" t="inlineStr">
+      <c r="I11" s="30" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J11" s="41" t="inlineStr">
+      <c r="J11" s="31" t="inlineStr">
         <is>
           <t>gunicorn pid 102228 + 4 workers</t>
         </is>
       </c>
-      <c r="K11" s="51" t="inlineStr">
+      <c r="K11" s="33" t="inlineStr">
         <is>
           <t>【场景】134 dev 验证完成，要给生产用上钉钉 OA 框架；【使用】promote_110.sh + 110 .env 启用 OA，admin 维护流程。</t>
         </is>
@@ -2255,24 +2352,24 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I12" s="53" t="inlineStr">
+      <c r="I12" s="30" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="J12" s="41" t="inlineStr">
+      <c r="J12" s="31" t="inlineStr">
         <is>
           <t>框架就绪、暂不启用</t>
         </is>
       </c>
-      <c r="K12" s="51" t="inlineStr">
+      <c r="K12" s="33" t="inlineStr">
         <is>
           <t>【场景】110 prod 先上框架、暂不启用；【使用】admin 维护 ext_approval_flow / policy，把 audit_driver 切到 dingtalk_oa 即可启用。</t>
         </is>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="35" t="inlineStr">
+      <c r="A13" s="36" t="inlineStr">
         <is>
           <t>gh-ost 无锁 DDL</t>
         </is>
@@ -2312,17 +2409,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I13" s="53" t="inlineStr">
+      <c r="I13" s="30" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="J13" s="41" t="inlineStr">
+      <c r="J13" s="31" t="inlineStr">
         <is>
           <t>docs/designs/...html</t>
         </is>
       </c>
-      <c r="K13" s="51" t="inlineStr">
+      <c r="K13" s="33" t="inlineStr">
         <is>
           <t>【场景】v0.3.0 要做什么 / 不做什么团队对齐；【使用】浏览器打开 docs/designs/2026-08-05_gh-ost-product-design.html，含场景、流程、验收标准。</t>
         </is>
@@ -2365,17 +2462,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I14" s="53" t="inlineStr">
+      <c r="I14" s="30" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="J14" s="41" t="inlineStr">
+      <c r="J14" s="31" t="inlineStr">
         <is>
           <t>/usr/local/bin/gh-ost</t>
         </is>
       </c>
-      <c r="K14" s="50" t="inlineStr">
+      <c r="K14" s="32" t="inlineStr">
         <is>
           <t>【场景】dev 环境演练无锁 DDL；【使用】gh-ost --version 验证 v1.1.10；后续 Archery 调它时走 settings.CUSTOM_GH_OST_BIN。</t>
         </is>
@@ -2418,17 +2515,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I15" s="53" t="inlineStr">
+      <c r="I15" s="30" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="J15" s="41" t="inlineStr">
+      <c r="J15" s="31" t="inlineStr">
         <is>
           <t>状态机 + 进度字段</t>
         </is>
       </c>
-      <c r="K15" s="51" t="inlineStr">
+      <c r="K15" s="33" t="inlineStr">
         <is>
           <t>【场景】gh-ost 任务需要持久化记录 + admin 可查；【使用】admin → 扩展表 → gh-ost 任务，能看每条 task 的状态/进度/进程/错误。</t>
         </is>
@@ -2471,17 +2568,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I16" s="53" t="inlineStr">
+      <c r="I16" s="30" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="J16" s="41" t="inlineStr">
+      <c r="J16" s="31" t="inlineStr">
         <is>
           <t>只读检查</t>
         </is>
       </c>
-      <c r="K16" s="51" t="inlineStr">
+      <c r="K16" s="33" t="inlineStr">
         <is>
           <t>【场景】防止 gh-ost 跑挂了（binlog 不对、磁盘不够、权限缺、SQL 不合法、源表不对）；【使用】业务方勾"启用 gh-ost"时自动跑，5/5 PASS 才允许起进程。</t>
         </is>
@@ -2524,17 +2621,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I17" s="53" t="inlineStr">
+      <c r="I17" s="30" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="J17" s="41" t="inlineStr">
+      <c r="J17" s="31" t="inlineStr">
         <is>
           <t>precheck/enable/start/cancel/status/progress</t>
         </is>
       </c>
-      <c r="K17" s="51" t="inlineStr">
+      <c r="K17" s="33" t="inlineStr">
         <is>
           <t>【场景】前后端交互 + 业务方看迁移进度；【使用】POST /gh_ost/{action}/&lt;wf_id&gt;/ 触发；GET /gh_ost/progress/&lt;wf_id&gt;/ 看可视化进度面板（3s 自动刷新）。</t>
         </is>
@@ -2577,17 +2674,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I18" s="53" t="inlineStr">
+      <c r="I18" s="30" t="inlineStr">
         <is>
           <t>0.3</t>
         </is>
       </c>
-      <c r="J18" s="41" t="inlineStr">
+      <c r="J18" s="31" t="inlineStr">
         <is>
           <t>4 bug</t>
         </is>
       </c>
-      <c r="K18" s="51" t="inlineStr">
+      <c r="K18" s="33" t="inlineStr">
         <is>
           <t>【场景】alpha 端到端要跑通；【使用】用户无感，自动修复 SqlWorkflowContent OneToOne / PARTITION_NAME 列名 / ENGINE 大小写 / .env 兜底直连。</t>
         </is>
@@ -2630,17 +2727,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I19" s="53" t="inlineStr">
+      <c r="I19" s="30" t="inlineStr">
         <is>
           <t>0.3</t>
         </is>
       </c>
-      <c r="J19" s="41" t="inlineStr">
+      <c r="J19" s="31" t="inlineStr">
         <is>
           <t>Popen + nohup</t>
         </is>
       </c>
-      <c r="K19" s="52" t="inlineStr">
+      <c r="K19" s="37" t="inlineStr">
         <is>
           <t>【场景】业务方提交 ALTER TABLE 工单要真改表；【使用】业务方在工单详情勾选 gh-ost → 5/5 PASS → DBA admin 点"启动"。</t>
         </is>
@@ -2683,17 +2780,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I20" s="53" t="inlineStr">
+      <c r="I20" s="30" t="inlineStr">
         <is>
           <t>0.3</t>
         </is>
       </c>
-      <c r="J20" s="41" t="inlineStr">
+      <c r="J20" s="31" t="inlineStr">
         <is>
           <t>1.1.10 输出兼容</t>
         </is>
       </c>
-      <c r="K20" s="51" t="inlineStr">
+      <c r="K20" s="33" t="inlineStr">
         <is>
           <t>【场景】gh-ost 进程输出要可视化；【使用】poller 自动每 3s 解析 log → 写 task.progress_* → 进度面板实时更新。</t>
         </is>
@@ -2736,17 +2833,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I21" s="53" t="inlineStr">
+      <c r="I21" s="30" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="J21" s="41" t="inlineStr">
+      <c r="J21" s="31" t="inlineStr">
         <is>
           <t>3s 轮询</t>
         </is>
       </c>
-      <c r="K21" s="51" t="inlineStr">
+      <c r="K21" s="33" t="inlineStr">
         <is>
           <t>【场景】gh-ost 跑完后状态要自动切到 success/failed；【使用】poller 检测进程死亡 + 解析 log 末尾 → 自动 _finalize_task 写终态。</t>
         </is>
@@ -2789,17 +2886,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I22" s="53" t="inlineStr">
+      <c r="I22" s="30" t="inlineStr">
         <is>
           <t>0.3</t>
         </is>
       </c>
-      <c r="J22" s="41" t="inlineStr">
+      <c r="J22" s="31" t="inlineStr">
         <is>
           <t>DBA 介入入口</t>
         </is>
       </c>
-      <c r="K22" s="52" t="inlineStr">
+      <c r="K22" s="37" t="inlineStr">
         <is>
           <t>【场景】DBA 紧急介入（取消/重试/回滚）；【使用】admin → gh-ost 任务 → 勾选 → 选 action（取消当前、重试失败、手动 drop 影子表）。</t>
         </is>
@@ -2842,17 +2939,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I23" s="53" t="inlineStr">
+      <c r="I23" s="30" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="J23" s="41" t="inlineStr">
+      <c r="J23" s="31" t="inlineStr">
         <is>
           <t>best-effort</t>
         </is>
       </c>
-      <c r="K23" s="52" t="inlineStr">
+      <c r="K23" s="37" t="inlineStr">
         <is>
           <t>【场景】DBA 群要知道工单迁移结果；【使用】配置 110 .env 的 DINGTALK_NOTIFY_WEBHOOK，task 终态时自动 @ 发起人 + 报告耗时。</t>
         </is>
@@ -2895,17 +2992,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I24" s="53" t="inlineStr">
+      <c r="I24" s="30" t="inlineStr">
         <is>
           <t>0.3</t>
         </is>
       </c>
-      <c r="J24" s="41" t="inlineStr">
+      <c r="J24" s="31" t="inlineStr">
         <is>
           <t>生产保护</t>
         </is>
       </c>
-      <c r="K24" s="51" t="inlineStr">
+      <c r="K24" s="33" t="inlineStr">
         <is>
           <t>【场景】生产高峰期不能压垮 MySQL；【使用】poller 每 10s 查 Threads_running → 超阈值 SIGSTOP gh-ost → 负载降下来 SIGCONT。</t>
         </is>
@@ -2948,17 +3045,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I25" s="53" t="inlineStr">
+      <c r="I25" s="30" t="inlineStr">
         <is>
           <t>0.3</t>
         </is>
       </c>
-      <c r="J25" s="41" t="inlineStr">
+      <c r="J25" s="31" t="inlineStr">
         <is>
           <t>管理命令</t>
         </is>
       </c>
-      <c r="K25" s="52" t="inlineStr">
+      <c r="K25" s="37" t="inlineStr">
         <is>
           <t>【场景】失败留下的影子表越攒越多；【使用】django-q 调度 /usr/bin/python manage.py cleanup_ghost_tables（或手动跑加 --dry-run 预览）。</t>
         </is>
@@ -3001,17 +3098,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I26" s="53" t="inlineStr">
+      <c r="I26" s="30" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="J26" s="41" t="inlineStr">
+      <c r="J26" s="31" t="inlineStr">
         <is>
           <t>5 次真改</t>
         </is>
       </c>
-      <c r="K26" s="52" t="inlineStr">
+      <c r="K26" s="37" t="inlineStr">
         <is>
           <t>【场景】验证端到端在真实业务表上能跑通；【使用】DBA 看 task 状态从 queued → running → success，影子表自动 drop。</t>
         </is>
@@ -3029,12 +3126,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D27" s="36" t="inlineStr">
+      <c r="D27" s="38" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="E27" s="34" t="inlineStr">
+      <c r="E27" s="35" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
@@ -3044,7 +3141,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G27" s="34" t="inlineStr">
+      <c r="G27" s="35" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -3054,17 +3151,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I27" s="53" t="inlineStr">
+      <c r="I27" s="30" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J27" s="42" t="inlineStr">
+      <c r="J27" s="39" t="inlineStr">
         <is>
           <t>等 webhook + 密文修复</t>
         </is>
       </c>
-      <c r="K27" s="52" t="inlineStr">
+      <c r="K27" s="37" t="inlineStr">
         <is>
           <t>【场景】dev 验证完要上生产；【使用】配 110 .env 配 DINGTALK_NOTIFY_WEBHOOK + DBA 重新保存 instance user/password（解 mirage 密文）+ promote_110.sh。</t>
         </is>
@@ -3082,12 +3179,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D28" s="36" t="inlineStr">
+      <c r="D28" s="38" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="E28" s="37" t="inlineStr">
+      <c r="E28" s="40" t="inlineStr">
         <is>
           <t>可选</t>
         </is>
@@ -3107,24 +3204,24 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I28" s="53" t="inlineStr">
+      <c r="I28" s="30" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="J28" s="42" t="inlineStr">
+      <c r="J28" s="39" t="inlineStr">
         <is>
           <t>5 行 diff</t>
         </is>
       </c>
-      <c r="K28" s="51" t="inlineStr">
+      <c r="K28" s="33" t="inlineStr">
         <is>
           <t>【场景】bigint 精度问题影响所有 1.14.0 用户；【使用】mavis PR 到 github.com/hhyo/Archery，5 行 diff（sql_api/renderers.py 加 bigint_as_string=True）。</t>
         </is>
       </c>
     </row>
     <row r="29" ht="48" customHeight="1">
-      <c r="A29" s="38" t="inlineStr">
+      <c r="A29" s="41" t="inlineStr">
         <is>
           <t>收尾</t>
         </is>
@@ -3139,12 +3236,12 @@
           <t>2026-08-12 后</t>
         </is>
       </c>
-      <c r="D29" s="36" t="inlineStr">
+      <c r="D29" s="38" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="E29" s="34" t="inlineStr">
+      <c r="E29" s="35" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
@@ -3164,17 +3261,17 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I29" s="53" t="inlineStr">
+      <c r="I29" s="30" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="J29" s="42" t="inlineStr">
+      <c r="J29" s="39" t="inlineStr">
         <is>
           <t>A 级回滚保险到期</t>
         </is>
       </c>
-      <c r="K29" s="52" t="inlineStr">
+      <c r="K29" s="37" t="inlineStr">
         <is>
           <t>【场景】110 prod 旧版保留 7 天后可以清；【使用】DBA 在 2026-08-12 后跑 rm -rf /dbdata/archery_v114/ + 删 /backup/promote/switch_20260805_201046/。</t>
         </is>
@@ -3192,12 +3289,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D30" s="36" t="inlineStr">
+      <c r="D30" s="38" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="E30" s="37" t="inlineStr">
+      <c r="E30" s="40" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
@@ -3207,7 +3304,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G30" s="39" t="inlineStr">
+      <c r="G30" s="42" t="inlineStr">
         <is>
           <t>高</t>
         </is>
@@ -3217,24 +3314,24 @@
           <t>马克群</t>
         </is>
       </c>
-      <c r="I30" s="49" t="inlineStr">
+      <c r="I30" s="43" t="inlineStr">
         <is>
           <t>5+</t>
         </is>
       </c>
-      <c r="J30" s="42" t="inlineStr">
+      <c r="J30" s="39" t="inlineStr">
         <is>
           <t>独立项目</t>
         </is>
       </c>
-      <c r="K30" s="52" t="inlineStr">
+      <c r="K30" s="37" t="inlineStr">
         <is>
           <t>【场景】5.7 已 EOL，必须升级到 8.0；【使用】独立项目评估 → 语法兼容性测试 + 字符集迁移 + 复制拓扑验证 → 切流（预计 5+ 天）。</t>
         </is>
       </c>
     </row>
     <row r="31" ht="48" customHeight="1">
-      <c r="A31" s="35" t="inlineStr">
+      <c r="A31" s="36" t="inlineStr">
         <is>
           <t>gh-ost 无锁 DDL</t>
         </is>
@@ -3244,536 +3341,921 @@
           <t>v0.4.0 列压缩</t>
         </is>
       </c>
-      <c r="C31" s="54" t="inlineStr">
+      <c r="C31" s="25" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="D31" s="55" t="inlineStr">
+      <c r="D31" s="26" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="E31" s="56" t="inlineStr">
+      <c r="E31" s="27" t="inlineStr">
         <is>
           <t>已发布</t>
         </is>
       </c>
-      <c r="F31" s="57" t="inlineStr">
+      <c r="F31" s="28" t="inlineStr">
         <is>
           <t>33cfd0f</t>
         </is>
       </c>
-      <c r="G31" s="58" t="inlineStr">
+      <c r="G31" s="35" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H31" s="59" t="inlineStr">
+      <c r="H31" s="44" t="inlineStr">
         <is>
           <t>mavis</t>
         </is>
       </c>
-      <c r="I31" s="53" t="inlineStr">
+      <c r="I31" s="30" t="inlineStr">
         <is>
           <t>0.3</t>
         </is>
       </c>
-      <c r="J31" s="60" t="inlineStr">
+      <c r="J31" s="45" t="inlineStr">
         <is>
           <t>Excel 列压缩到 11 列；DROP COLUMN + ADD COLUMN 改写为单行 ALTER 链</t>
         </is>
       </c>
-      <c r="K31" s="61" t="inlineStr">
+      <c r="K31" s="46" t="inlineStr">
         <is>
           <t>【场景】v0.3.0 之前 DROP/ADD 拆成两条工单，134 dev 演练 1 张表要走 2 次 gh-ost。【使用】工单页面检测到 DROP+ADD 同表同提交 → 合并成 `ALTER TABLE x DROP col_a, ADD col_b` 单条 → 1 次 gh-ost 完成。</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="48" customHeight="1">
-      <c r="A32" s="33" t="inlineStr">
+    <row r="32" ht="56" customHeight="1">
+      <c r="A32" s="57" t="inlineStr">
+        <is>
+          <t>gh-ost 无锁 DDL</t>
+        </is>
+      </c>
+      <c r="B32" s="58" t="inlineStr">
+        <is>
+          <t>v0.4.1-alpha：ArchiveConfig 加进度字段（last_archive_status + progress_pct）</t>
+        </is>
+      </c>
+      <c r="C32" s="59" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D32" s="60" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E32" s="61" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="F32" s="62" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="G32" s="63" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H32" s="64" t="inlineStr">
+        <is>
+          <t>mavis</t>
+        </is>
+      </c>
+      <c r="I32" s="65" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J32" s="66" t="inlineStr">
+        <is>
+          <t>admin list_display 加 last_archive_status / progress_pct 字段</t>
+        </is>
+      </c>
+      <c r="K32" s="67" t="inlineStr">
+        <is>
+          <t>【场景】现有 archive_config 表只有 last_archive_time，看不到归档是否成功、跑了多少行。【使用】新增字段 last_archive_status（success/failed/running/pending）+ progress_pct + rows_archived；admin 列表直接看到状态。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="56" customHeight="1">
+      <c r="A33" s="57" t="inlineStr">
+        <is>
+          <t>gh-ost 无锁 DDL</t>
+        </is>
+      </c>
+      <c r="B33" s="58" t="inlineStr">
+        <is>
+          <t>v0.4.1-alpha：归档详情页增强（archive_detail.html 进度条 + 历史日志表格）</t>
+        </is>
+      </c>
+      <c r="C33" s="59" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D33" s="60" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E33" s="61" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="F33" s="62" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="G33" s="61" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H33" s="64" t="inlineStr">
+        <is>
+          <t>mavis</t>
+        </is>
+      </c>
+      <c r="I33" s="65" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J33" s="66" t="inlineStr">
+        <is>
+          <t>templates/sqlarchive.html 改造 + ArchiveLog 表格化</t>
+        </is>
+      </c>
+      <c r="K33" s="67" t="inlineStr">
+        <is>
+          <t>【场景】DBA 点进归档详情只看到基础字段，看不到每次归档跑了多少行 / 用了多久 / 失败原因。【使用】详情页加 进度条 + 历史日志表格（select_cnt/insert_cnt/delete_cnt/start_time/end_time/success/error_info）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="56" customHeight="1">
+      <c r="A34" s="57" t="inlineStr">
+        <is>
+          <t>gh-ost 无锁 DDL</t>
+        </is>
+      </c>
+      <c r="B34" s="58" t="inlineStr">
+        <is>
+          <t>v0.4.1-alpha：归档完成钉钉通知（ArchiveLog 写完后发）</t>
+        </is>
+      </c>
+      <c r="C34" s="59" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D34" s="60" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E34" s="61" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="F34" s="62" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="G34" s="63" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H34" s="64" t="inlineStr">
+        <is>
+          <t>mavis</t>
+        </is>
+      </c>
+      <c r="I34" s="65" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J34" s="66" t="inlineStr">
+        <is>
+          <t>archiver.archive() 末尾 async_task 发钉钉群</t>
+        </is>
+      </c>
+      <c r="K34" s="67" t="inlineStr">
+        <is>
+          <t>【场景】归档是异步任务，DBA 不盯着页面不知道跑完没。【使用】archive() 完成后 async_task 调 notify_terminal，发钉钉群（best-effort，webhook 没配就 skip）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="56" customHeight="1">
+      <c r="A35" s="57" t="inlineStr">
+        <is>
+          <t>gh-ost 无锁 DDL</t>
+        </is>
+      </c>
+      <c r="B35" s="58" t="inlineStr">
+        <is>
+          <t>v0.4.2-alpha：ArchiveConfig 加 auto_rebuild_after_archive 字段 + 归档完成 hook</t>
+        </is>
+      </c>
+      <c r="C35" s="59" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D35" s="60" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E35" s="61" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="F35" s="62" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="G35" s="61" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H35" s="64" t="inlineStr">
+        <is>
+          <t>mavis</t>
+        </is>
+      </c>
+      <c r="I35" s="65" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J35" s="66" t="inlineStr">
+        <is>
+          <t>Boolean 字段；archive() 成功后自动触发 v0.4.5 rebuild task</t>
+        </is>
+      </c>
+      <c r="K35" s="67" t="inlineStr">
+        <is>
+          <t>【场景】归档删完数据后表会有大量碎片，需要 OPTIMIZE/重建。以前是手动两步走。【使用】ArchiveConfig 加 auto_rebuild_after_archive Boolean（默认 False）；archive() 成功后检测字段 → 写 DdlGhostTask（task_type=rebuild, related_task_id=archive_id）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="56" customHeight="1">
+      <c r="A36" s="57" t="inlineStr">
+        <is>
+          <t>gh-ost 无锁 DDL</t>
+        </is>
+      </c>
+      <c r="B36" s="58" t="inlineStr">
+        <is>
+          <t>v0.4.2-beta：134 dev 演练归档→自动回收（accesscard_black_detail 造数据）</t>
+        </is>
+      </c>
+      <c r="C36" s="59" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D36" s="60" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E36" s="61" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="F36" s="62" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="G36" s="61" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H36" s="64" t="inlineStr">
+        <is>
+          <t>mavis</t>
+        </is>
+      </c>
+      <c r="I36" s="65" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J36" s="66" t="inlineStr">
+        <is>
+          <t>134 dev 演练：归档 100 万行历史数据 → 验证自动 rebuild</t>
+        </is>
+      </c>
+      <c r="K36" s="67" t="inlineStr">
+        <is>
+          <t>【场景】真实业务表测归档+重建联动。【使用】DBA 在 134 dev archery_dev 库 accesscard_black_detail 灌 100 万行 → 配归档+勾 auto_rebuild → 触发归档 → 验证 rebuild 自动跑 + 碎片回收成功。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="56" customHeight="1">
+      <c r="A37" s="57" t="inlineStr">
+        <is>
+          <t>gh-ost 无锁 DDL</t>
+        </is>
+      </c>
+      <c r="B37" s="58" t="inlineStr">
+        <is>
+          <t>v0.4.3-alpha：ArchiveLog 前端表格化（select/insert/delete 数量可视化）</t>
+        </is>
+      </c>
+      <c r="C37" s="59" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D37" s="60" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E37" s="61" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="F37" s="62" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="G37" s="63" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H37" s="64" t="inlineStr">
+        <is>
+          <t>mavis</t>
+        </is>
+      </c>
+      <c r="I37" s="65" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J37" s="66" t="inlineStr">
+        <is>
+          <t>archive_log.html 加可视化（条形图 / 数字徽章）</t>
+        </is>
+      </c>
+      <c r="K37" s="67" t="inlineStr">
+        <is>
+          <t>【场景】归档日志表里只有 select_cnt/insert_cnt/delete_cnt 三个数字，肉眼比对累。【使用】前端加条形图 + 颜色徽章（成功=绿/失败=红），DBA 一眼看成功率和数据量趋势。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="56" customHeight="1">
+      <c r="A38" s="57" t="inlineStr">
+        <is>
+          <t>gh-ost 无锁 DDL</t>
+        </is>
+      </c>
+      <c r="B38" s="58" t="inlineStr">
+        <is>
+          <t>v0.4.3-alpha：归档成功率统计 dashboard（周/月）</t>
+        </is>
+      </c>
+      <c r="C38" s="59" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D38" s="60" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E38" s="61" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="F38" s="62" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="G38" s="63" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H38" s="64" t="inlineStr">
+        <is>
+          <t>mavis</t>
+        </is>
+      </c>
+      <c r="I38" s="65" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J38" s="66" t="inlineStr">
+        <is>
+          <t>dashboard 模块加 archive 统计卡片</t>
+        </is>
+      </c>
+      <c r="K38" s="67" t="inlineStr">
+        <is>
+          <t>【场景】DBA 主管要看全局归档健康度。【使用】dashboard 加卡片：本周归档次数 / 成功率 / 总归档行数 / 失败 Top 5。SQL 用 SUM/COUNT GROUP BY week，django 模板渲染。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="56" customHeight="1">
+      <c r="A39" s="77" t="inlineStr">
         <is>
           <t>钉钉 OA 集成</t>
         </is>
       </c>
-      <c r="B32" s="25" t="inlineStr">
+      <c r="B39" s="25" t="inlineStr">
         <is>
           <t>v0.2.1 钉钉 OA 模板（process_code）</t>
         </is>
       </c>
-      <c r="C32" s="25" t="inlineStr">
+      <c r="C39" s="25" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="D32" s="36" t="inlineStr">
+      <c r="D39" s="38" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="E32" s="34" t="inlineStr">
+      <c r="E39" s="35" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="F32" s="28" t="inlineStr">
+      <c r="F39" s="28" t="inlineStr">
         <is>
           <t>DRAFT</t>
         </is>
       </c>
-      <c r="G32" s="34" t="inlineStr">
+      <c r="G39" s="35" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H32" s="29" t="inlineStr">
+      <c r="H39" s="29" t="inlineStr">
         <is>
           <t>马克群</t>
         </is>
       </c>
-      <c r="I32" s="53" t="inlineStr">
+      <c r="I39" s="30" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="J32" s="43" t="inlineStr">
+      <c r="J39" s="48" t="inlineStr">
         <is>
           <t>未开始；用户在 oa.dingtalk.com 建模板</t>
         </is>
       </c>
-      <c r="K32" s="50" t="inlineStr"/>
-    </row>
-    <row r="33" ht="24" customHeight="1">
-      <c r="A33" s="33" t="inlineStr">
+      <c r="K39" s="32" t="inlineStr"/>
+    </row>
+    <row r="40" ht="56" customHeight="1">
+      <c r="A40" s="77" t="inlineStr">
         <is>
           <t>钉钉 OA 集成</t>
         </is>
       </c>
-      <c r="B33" s="25" t="inlineStr">
+      <c r="B40" s="25" t="inlineStr">
         <is>
           <t>v0.2.2 Tunnel + 回调加密（cloudflared）</t>
         </is>
       </c>
-      <c r="C33" s="25" t="inlineStr">
+      <c r="C40" s="25" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="D33" s="36" t="inlineStr">
+      <c r="D40" s="38" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="E33" s="34" t="inlineStr">
+      <c r="E40" s="35" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="F33" s="28" t="inlineStr">
+      <c r="F40" s="28" t="inlineStr">
         <is>
           <t>DRAFT</t>
         </is>
       </c>
-      <c r="G33" s="34" t="inlineStr">
+      <c r="G40" s="35" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H33" s="29" t="inlineStr">
+      <c r="H40" s="29" t="inlineStr">
         <is>
           <t>马克群</t>
         </is>
       </c>
-      <c r="I33" s="53" t="inlineStr">
+      <c r="I40" s="30" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J33" s="43" t="inlineStr">
+      <c r="J40" s="48" t="inlineStr">
         <is>
           <t>前置条件：DBA 需自备域名（公网已备案），不能用 trycloudflare 临时域名；callback URL 走域名 + HTTPS</t>
         </is>
       </c>
-      <c r="K33" s="50" t="inlineStr"/>
-    </row>
-    <row r="34" ht="24" customHeight="1">
-      <c r="A34" s="33" t="inlineStr">
+      <c r="K40" s="32" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="77" t="inlineStr">
         <is>
           <t>钉钉 OA 集成</t>
         </is>
       </c>
-      <c r="B34" s="25" t="inlineStr">
+      <c r="B41" s="25" t="inlineStr">
         <is>
           <t>v0.2.3 对账 cron + runbook</t>
         </is>
       </c>
-      <c r="C34" s="25" t="inlineStr">
+      <c r="C41" s="25" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="D34" s="36" t="inlineStr">
+      <c r="D41" s="38" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="E34" s="34" t="inlineStr">
+      <c r="E41" s="35" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="F34" s="28" t="inlineStr">
+      <c r="F41" s="28" t="inlineStr">
         <is>
           <t>DRAFT</t>
         </is>
       </c>
-      <c r="G34" s="34" t="inlineStr">
+      <c r="G41" s="35" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H34" s="29" t="inlineStr">
+      <c r="H41" s="29" t="inlineStr">
         <is>
           <t>马克群</t>
         </is>
       </c>
-      <c r="I34" s="53" t="inlineStr">
+      <c r="I41" s="30" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J34" s="43" t="inlineStr">
+      <c r="J41" s="48" t="inlineStr">
         <is>
           <t>依赖：v0.2.1 模板 + v0.2.2 tunnel 都完成后才能做（callback 不通就没法对账）</t>
         </is>
       </c>
-      <c r="K34" s="50" t="inlineStr"/>
-    </row>
-    <row r="35" ht="56" customHeight="1">
-      <c r="A35" s="62" t="inlineStr">
+      <c r="K41" s="32" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="57" t="inlineStr">
         <is>
           <t>gh-ost 无锁 DDL</t>
         </is>
       </c>
-      <c r="B35" s="63" t="inlineStr">
+      <c r="B42" s="25" t="inlineStr">
         <is>
           <t>v0.4.5-alpha：model 改造（task_type + target_table + 拆 OneToOne）</t>
         </is>
       </c>
-      <c r="C35" s="64" t="inlineStr">
+      <c r="C42" s="52" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D35" s="65" t="inlineStr">
+      <c r="D42" s="38" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="E35" s="58" t="inlineStr">
+      <c r="E42" s="35" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="F35" s="66" t="inlineStr">
+      <c r="F42" s="53" t="inlineStr">
         <is>
           <t>DRAFT</t>
         </is>
       </c>
-      <c r="G35" s="58" t="inlineStr">
+      <c r="G42" s="35" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H35" s="59" t="inlineStr">
-        <is>
-          <t>mavis</t>
-        </is>
-      </c>
-      <c r="I35" s="53" t="n">
+      <c r="H42" s="29" t="inlineStr">
+        <is>
+          <t>马克群</t>
+        </is>
+      </c>
+      <c r="I42" s="30" t="n">
         <v>0.3</v>
       </c>
-      <c r="J35" s="67" t="inlineStr">
+      <c r="J42" s="54" t="inlineStr">
         <is>
           <t>拆 OneToOne 为 ForeignKey(null)；task_type 区分 ghost/rebuild；Meta.unique_together 约束</t>
         </is>
       </c>
-      <c r="K35" s="50" t="inlineStr">
+      <c r="K42" s="32" t="inlineStr">
         <is>
           <t>【场景】ghost 是工单级（OneToOne SqlWorkflow），rebuild 是表级（DBA 手动选表）。【使用】新增字段 `task_type`/`target_table`/`related_task_id`；rebuild 时 workflow=NULL，target_table 存 `db.table`。</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="56" customHeight="1">
-      <c r="A36" s="62" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="57" t="inlineStr">
         <is>
           <t>gh-ost 无锁 DDL</t>
         </is>
       </c>
-      <c r="B36" s="63" t="inlineStr">
+      <c r="B43" s="25" t="inlineStr">
         <is>
           <t>v0.4.5-alpha：rebuild service（services/rebuild.py）</t>
         </is>
       </c>
-      <c r="C36" s="64" t="inlineStr">
+      <c r="C43" s="52" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D36" s="65" t="inlineStr">
+      <c r="D43" s="38" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="E36" s="58" t="inlineStr">
+      <c r="E43" s="35" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="F36" s="66" t="inlineStr">
+      <c r="F43" s="53" t="inlineStr">
         <is>
           <t>DRAFT</t>
         </is>
       </c>
-      <c r="G36" s="56" t="inlineStr">
+      <c r="G43" s="27" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="H36" s="59" t="inlineStr">
-        <is>
-          <t>mavis</t>
-        </is>
-      </c>
-      <c r="I36" s="53" t="n">
+      <c r="H43" s="29" t="inlineStr">
+        <is>
+          <t>马克群</t>
+        </is>
+      </c>
+      <c r="I43" s="30" t="n">
         <v>0.3</v>
       </c>
-      <c r="J36" s="67" t="inlineStr">
+      <c r="J43" s="54" t="inlineStr">
         <is>
           <t>复用 runner.py，差别只在 --alter 改 COMMENT 空 alter 触发重建</t>
         </is>
       </c>
-      <c r="K36" s="50" t="inlineStr">
+      <c r="K43" s="32" t="inlineStr">
         <is>
           <t>【场景】大表碎片率高，OPTIMIZE TABLE 锁表；pt-osc 装新环境成本高。【使用】gh-ost 跑 `ALTER TABLE x COMMENT 'archery-auto-rebuild-YYYYMMDD'`，结构不变触发表重建，几秒锁表完成。</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="56" customHeight="1">
-      <c r="A37" s="62" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="57" t="inlineStr">
         <is>
           <t>gh-ost 无锁 DDL</t>
         </is>
       </c>
-      <c r="B37" s="63" t="inlineStr">
+      <c r="B44" s="25" t="inlineStr">
         <is>
           <t>v0.4.5-alpha：视图 + 路由（rebuild/list 端点）</t>
         </is>
       </c>
-      <c r="C37" s="64" t="inlineStr">
+      <c r="C44" s="52" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D37" s="65" t="inlineStr">
+      <c r="D44" s="38" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="E37" s="58" t="inlineStr">
+      <c r="E44" s="35" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="F37" s="66" t="inlineStr">
+      <c r="F44" s="53" t="inlineStr">
         <is>
           <t>DRAFT</t>
         </is>
       </c>
-      <c r="G37" s="58" t="inlineStr">
+      <c r="G44" s="35" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H37" s="59" t="inlineStr">
-        <is>
-          <t>mavis</t>
-        </is>
-      </c>
-      <c r="I37" s="53" t="n">
+      <c r="H44" s="29" t="inlineStr">
+        <is>
+          <t>马克群</t>
+        </is>
+      </c>
+      <c r="I44" s="30" t="n">
         <v>0.3</v>
       </c>
-      <c r="J37" s="67" t="inlineStr">
+      <c r="J44" s="54" t="inlineStr">
         <is>
           <t>新增 POST /gh_ost/rebuild/&lt;table_id&gt;/ + GET /gh_ost/rebuild/list/</t>
         </is>
       </c>
-      <c r="K37" s="50" t="inlineStr">
+      <c r="K44" s="32" t="inlineStr">
         <is>
           <t>【场景】DBA 选 instance + 表 → 一键触发 rebuild。【使用】DBA 在 admin 表列表点 "重建" → 写 task（task_type=rebuild, workflow=NULL）→ 启动 gh-ost → 进度面板 polling 3s。</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="56" customHeight="1">
-      <c r="A38" s="62" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="57" t="inlineStr">
         <is>
           <t>gh-ost 无锁 DDL</t>
         </is>
       </c>
-      <c r="B38" s="63" t="inlineStr">
+      <c r="B45" s="25" t="inlineStr">
         <is>
           <t>v0.4.5-alpha：admin + UI（list_filter + 批量 action）</t>
         </is>
       </c>
-      <c r="C38" s="64" t="inlineStr">
+      <c r="C45" s="52" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D38" s="65" t="inlineStr">
+      <c r="D45" s="38" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="E38" s="58" t="inlineStr">
+      <c r="E45" s="35" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="F38" s="66" t="inlineStr">
+      <c r="F45" s="53" t="inlineStr">
         <is>
           <t>DRAFT</t>
         </is>
       </c>
-      <c r="G38" s="58" t="inlineStr">
+      <c r="G45" s="35" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H38" s="59" t="inlineStr">
-        <is>
-          <t>mavis</t>
-        </is>
-      </c>
-      <c r="I38" s="53" t="n">
+      <c r="H45" s="29" t="inlineStr">
+        <is>
+          <t>马克群</t>
+        </is>
+      </c>
+      <c r="I45" s="30" t="n">
         <v>0.3</v>
       </c>
-      <c r="J38" s="67" t="inlineStr">
+      <c r="J45" s="54" t="inlineStr">
         <is>
           <t>admin list_filter 加 task_type；admin action 加 "批量重建"；progress.html 适配 rebuild 无工单场景</t>
         </is>
       </c>
-      <c r="K38" s="50" t="inlineStr">
+      <c r="K45" s="32" t="inlineStr">
         <is>
           <t>【场景】DBA 看到一堆要重建的表，挨个点太慢。【使用】admin 勾选 N 张表 → action 选 "批量重建" → 一次触发 N 个 rebuild task（按表排队，同表只跑 1 个）。</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="56" customHeight="1">
-      <c r="A39" s="62" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="57" t="inlineStr">
         <is>
           <t>gh-ost 无锁 DDL</t>
         </is>
       </c>
-      <c r="B39" s="63" t="inlineStr">
+      <c r="B46" s="25" t="inlineStr">
         <is>
           <t>v0.4.5-alpha：排队 + 关联归档（services/queue.py）</t>
         </is>
       </c>
-      <c r="C39" s="64" t="inlineStr">
+      <c r="C46" s="52" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D39" s="65" t="inlineStr">
+      <c r="D46" s="38" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="E39" s="58" t="inlineStr">
+      <c r="E46" s="35" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="F39" s="66" t="inlineStr">
+      <c r="F46" s="53" t="inlineStr">
         <is>
           <t>DRAFT</t>
         </is>
       </c>
-      <c r="G39" s="58" t="inlineStr">
+      <c r="G46" s="35" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H39" s="59" t="inlineStr">
-        <is>
-          <t>mavis</t>
-        </is>
-      </c>
-      <c r="I39" s="53" t="n">
+      <c r="H46" s="29" t="inlineStr">
+        <is>
+          <t>马克群</t>
+        </is>
+      </c>
+      <c r="I46" s="30" t="n">
         <v>0.5</v>
       </c>
-      <c r="J39" s="67" t="inlineStr">
+      <c r="J46" s="54" t="inlineStr">
         <is>
           <t>同表冲突排队（FIFO）；归档联动 auto_link_archive opt-in 开关</t>
         </is>
       </c>
-      <c r="K39" s="50" t="inlineStr">
+      <c r="K46" s="32" t="inlineStr">
         <is>
           <t>【场景】DBA 同时点 "归档 + 回收"，同表 2 个 task 撞车。【使用】rebuild 检测到同表有归档 task running → 排队等前面完成 → 归档完自动启动 rebuild。归档联动默认关，要开显式勾 "归档完自动回收"。</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="56" customHeight="1">
-      <c r="A40" s="62" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="57" t="inlineStr">
         <is>
           <t>gh-ost 无锁 DDL</t>
         </is>
       </c>
-      <c r="B40" s="63" t="inlineStr">
+      <c r="B47" s="25" t="inlineStr">
         <is>
           <t>v0.4.5-alpha：134 dev 演练（accesscard_black_detail 造碎片 → 重建）</t>
         </is>
       </c>
-      <c r="C40" s="64" t="inlineStr">
+      <c r="C47" s="52" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D40" s="65" t="inlineStr">
+      <c r="D47" s="38" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="E40" s="58" t="inlineStr">
+      <c r="E47" s="35" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="F40" s="66" t="inlineStr">
+      <c r="F47" s="53" t="inlineStr">
         <is>
           <t>DRAFT</t>
         </is>
       </c>
-      <c r="G40" s="58" t="inlineStr">
+      <c r="G47" s="35" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H40" s="59" t="inlineStr">
-        <is>
-          <t>mavis</t>
-        </is>
-      </c>
-      <c r="I40" s="53" t="n">
+      <c r="H47" s="29" t="inlineStr">
+        <is>
+          <t>马克群</t>
+        </is>
+      </c>
+      <c r="I47" s="30" t="n">
         <v>0.4</v>
       </c>
-      <c r="J40" s="67" t="inlineStr">
+      <c r="J47" s="54" t="inlineStr">
         <is>
           <t>删 50% 数据造碎片 → 跑 rebuild → 前后对比 INFORMATION_SCHEMA.TABLES.DATA_FREE</t>
         </is>
       </c>
-      <c r="K40" s="50" t="inlineStr">
+      <c r="K47" s="32" t="inlineStr">
         <is>
           <t>【场景】真实业务表测碎片回收效果。【使用】DBA 在 134 dev dev 库演练大表 accesscard_black_detail 上删一半行 → 点重建 → 观察 gh-ost 进度 → 验证 DATA_FREE 下降。重复 1 表 N 次验证限频 1 次/天/表。</t>
         </is>
@@ -3857,7 +4339,7 @@
         <f>COUNTIFS(功能开发计划!A:A,A5,功能开发计划!E:E,"已发布")</f>
         <v/>
       </c>
-      <c r="D5" s="44">
+      <c r="D5" s="72">
         <f>IFERROR(C5/B5,0)</f>
         <v/>
       </c>
@@ -3865,7 +4347,7 @@
         <f>COUNTIFS(功能开发计划!A:A,A5,功能开发计划!G:G,"高")</f>
         <v/>
       </c>
-      <c r="F5" s="45">
+      <c r="F5" s="73">
         <f>SUMPRODUCT((功能开发计划!A2:A33=A5)*ISNUMBER(功能开发计划!I2:I33)*功能开发计划!I2:I33)</f>
         <v/>
       </c>
@@ -3884,7 +4366,7 @@
         <f>COUNTIFS(功能开发计划!A:A,A6,功能开发计划!E:E,"已发布")</f>
         <v/>
       </c>
-      <c r="D6" s="44">
+      <c r="D6" s="72">
         <f>IFERROR(C6/B6,0)</f>
         <v/>
       </c>
@@ -3892,7 +4374,7 @@
         <f>COUNTIFS(功能开发计划!A:A,A6,功能开发计划!G:G,"高")</f>
         <v/>
       </c>
-      <c r="F6" s="45">
+      <c r="F6" s="73">
         <f>SUMPRODUCT((功能开发计划!A2:A33=A6)*ISNUMBER(功能开发计划!I2:I33)*功能开发计划!I2:I33)</f>
         <v/>
       </c>
@@ -3911,7 +4393,7 @@
         <f>COUNTIFS(功能开发计划!A:A,A7,功能开发计划!E:E,"已发布")</f>
         <v/>
       </c>
-      <c r="D7" s="44">
+      <c r="D7" s="72">
         <f>IFERROR(C7/B7,0)</f>
         <v/>
       </c>
@@ -3919,7 +4401,7 @@
         <f>COUNTIFS(功能开发计划!A:A,A7,功能开发计划!G:G,"高")</f>
         <v/>
       </c>
-      <c r="F7" s="45">
+      <c r="F7" s="73">
         <f>SUMPRODUCT((功能开发计划!A2:A33=A7)*ISNUMBER(功能开发计划!I2:I33)*功能开发计划!I2:I33)</f>
         <v/>
       </c>
@@ -3938,7 +4420,7 @@
         <f>COUNTIFS(功能开发计划!A:A,A8,功能开发计划!E:E,"已发布")</f>
         <v/>
       </c>
-      <c r="D8" s="44">
+      <c r="D8" s="72">
         <f>IFERROR(C8/B8,0)</f>
         <v/>
       </c>
@@ -3946,7 +4428,7 @@
         <f>COUNTIFS(功能开发计划!A:A,A8,功能开发计划!G:G,"高")</f>
         <v/>
       </c>
-      <c r="F8" s="45">
+      <c r="F8" s="73">
         <f>SUMPRODUCT((功能开发计划!A2:A33=A8)*ISNUMBER(功能开发计划!I2:I33)*功能开发计划!I2:I33)</f>
         <v/>
       </c>
@@ -3965,7 +4447,7 @@
         <f>SUM(C5:C8)</f>
         <v/>
       </c>
-      <c r="D9" s="46">
+      <c r="D9" s="74">
         <f>IFERROR(C9/B9,0)</f>
         <v/>
       </c>
@@ -3973,7 +4455,7 @@
         <f>SUM(E5:E8)</f>
         <v/>
       </c>
-      <c r="F9" s="47">
+      <c r="F9" s="75">
         <f>SUM(F5:F8)</f>
         <v/>
       </c>
@@ -3995,7 +4477,7 @@
           <t>总投入人天（已交付）</t>
         </is>
       </c>
-      <c r="B12" s="48">
+      <c r="B12" s="76">
         <f>SUMPRODUCT((功能开发计划!E2:E33="已发布")*ISNUMBER(功能开发计划!I2:I33)*功能开发计划!I2:I33)</f>
         <v/>
       </c>
@@ -4149,7 +4631,7 @@
         <f>COUNTIFS(功能开发计划!H:H,"mavis",功能开发计划!E:E,"待办")</f>
         <v/>
       </c>
-      <c r="D4" s="45">
+      <c r="D4" s="73">
         <f>SUMPRODUCT((功能开发计划!H2:H33="mavis")*(功能开发计划!E2:E33="已发布")*ISNUMBER(功能开发计划!I2:I33)*功能开发计划!I2:I33)</f>
         <v/>
       </c>
@@ -4168,7 +4650,7 @@
         <f>COUNTIFS(功能开发计划!H:H,"阿达叔叔",功能开发计划!E:E,"待办")</f>
         <v/>
       </c>
-      <c r="D5" s="45">
+      <c r="D5" s="73">
         <f>SUMPRODUCT((功能开发计划!H2:H33="阿达叔叔")*(功能开发计划!E2:E33="已发布")*ISNUMBER(功能开发计划!I2:I33)*功能开发计划!I2:I33)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
docs(reports): v0.4.5-alpha model 改造 commit 1 标已发布
- row 42 v0.4.5-alpha model 改造：100% / 已发布 / commit 6412da4
- 备注：134 dev makemigrations --check 0 missing + migrate --check 0 阻塞
- 134 dev 出口 443 受限，force push 后 134 dev fetch 失败，
  但 Django 自动生成的 migration 内容已落地 dev 仓库 working tree

CHANGELOG: docs/changelogs/2026-08-06_gh-ost-v045-alpha-skeleton.md
</commit_message>
<xml_diff>
--- a/docs/reports/2026-08-06_功能开发计划_v3.xlsx
+++ b/docs/reports/2026-08-06_功能开发计划_v3.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="55">
+  <fonts count="56">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -399,8 +399,13 @@
       <color rgb="0014171E"/>
       <sz val="9.5"/>
     </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="003A4256"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="54">
+  <fills count="55">
     <fill>
       <patternFill/>
     </fill>
@@ -709,6 +714,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FAF8F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F0EA"/>
       </patternFill>
     </fill>
   </fills>
@@ -1074,7 +1084,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1287,6 +1297,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="46" fillId="51" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="49" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="54" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3942,24 +3961,24 @@
           <t>v0.4.5-alpha：model 改造（task_type + target_table + 拆 OneToOne）</t>
         </is>
       </c>
-      <c r="C42" s="52" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D42" s="38" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="E42" s="35" t="inlineStr">
-        <is>
-          <t>待办</t>
-        </is>
-      </c>
-      <c r="F42" s="53" t="inlineStr">
-        <is>
-          <t>DRAFT</t>
+      <c r="C42" s="59" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D42" s="78" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E42" s="63" t="inlineStr">
+        <is>
+          <t>已发布</t>
+        </is>
+      </c>
+      <c r="F42" s="79" t="inlineStr">
+        <is>
+          <t>6412da4</t>
         </is>
       </c>
       <c r="G42" s="35" t="inlineStr">
@@ -3975,9 +3994,9 @@
       <c r="I42" s="30" t="n">
         <v>0.3</v>
       </c>
-      <c r="J42" s="54" t="inlineStr">
-        <is>
-          <t>拆 OneToOne 为 ForeignKey(null)；task_type 区分 ghost/rebuild；Meta.unique_together 约束</t>
+      <c r="J42" s="80" t="inlineStr">
+        <is>
+          <t>alpha 6 件第 1 件；134 dev makemigrations --check 0 missing + migrate --check 0 阻塞</t>
         </is>
       </c>
       <c r="K42" s="32" t="inlineStr">

</xml_diff>

<commit_message>
docs(reports): v0.4.5-alpha rebuild service commit 2 标已发布
</commit_message>
<xml_diff>
--- a/docs/reports/2026-08-06_功能开发计划_v3.xlsx
+++ b/docs/reports/2026-08-06_功能开发计划_v3.xlsx
@@ -4016,24 +4016,24 @@
           <t>v0.4.5-alpha：rebuild service（services/rebuild.py）</t>
         </is>
       </c>
-      <c r="C43" s="52" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D43" s="38" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="E43" s="35" t="inlineStr">
-        <is>
-          <t>待办</t>
-        </is>
-      </c>
-      <c r="F43" s="53" t="inlineStr">
-        <is>
-          <t>DRAFT</t>
+      <c r="C43" s="59" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D43" s="78" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E43" s="63" t="inlineStr">
+        <is>
+          <t>已发布</t>
+        </is>
+      </c>
+      <c r="F43" s="79" t="inlineStr">
+        <is>
+          <t>e8b2cf3</t>
         </is>
       </c>
       <c r="G43" s="27" t="inlineStr">
@@ -4049,9 +4049,9 @@
       <c r="I43" s="30" t="n">
         <v>0.3</v>
       </c>
-      <c r="J43" s="54" t="inlineStr">
-        <is>
-          <t>复用 runner.py，差别只在 --alter 改 COMMENT 空 alter 触发重建</t>
+      <c r="J43" s="80" t="inlineStr">
+        <is>
+          <t>重构 runner.build_ghost_command 加 rebuild_mode + 新建 rebuild.py；alter 改空 COMMENT 触发表重建</t>
         </is>
       </c>
       <c r="K43" s="32" t="inlineStr">

</xml_diff>

<commit_message>
docs(reports): v0.4.5-alpha views+路由 commit 3 标已发布
</commit_message>
<xml_diff>
--- a/docs/reports/2026-08-06_功能开发计划_v3.xlsx
+++ b/docs/reports/2026-08-06_功能开发计划_v3.xlsx
@@ -4071,24 +4071,24 @@
           <t>v0.4.5-alpha：视图 + 路由（rebuild/list 端点）</t>
         </is>
       </c>
-      <c r="C44" s="52" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D44" s="38" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="E44" s="35" t="inlineStr">
-        <is>
-          <t>待办</t>
-        </is>
-      </c>
-      <c r="F44" s="53" t="inlineStr">
-        <is>
-          <t>DRAFT</t>
+      <c r="C44" s="59" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D44" s="78" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E44" s="63" t="inlineStr">
+        <is>
+          <t>已发布</t>
+        </is>
+      </c>
+      <c r="F44" s="79" t="inlineStr">
+        <is>
+          <t>52b875b</t>
         </is>
       </c>
       <c r="G44" s="35" t="inlineStr">
@@ -4104,9 +4104,9 @@
       <c r="I44" s="30" t="n">
         <v>0.3</v>
       </c>
-      <c r="J44" s="54" t="inlineStr">
-        <is>
-          <t>新增 POST /gh_ost/rebuild/&lt;table_id&gt;/ + GET /gh_ost/rebuild/list/</t>
+      <c r="J44" s="80" t="inlineStr">
+        <is>
+          <t>新增 GET /gh_ost/rebuild/list/ + POST /gh_ost/rebuild/start/；同表冲突 alpha 阶段 409 拒绝</t>
         </is>
       </c>
       <c r="K44" s="32" t="inlineStr">

</xml_diff>

<commit_message>
docs(reports): v0.4.5-alpha admin+UI commit 4 标已发布
</commit_message>
<xml_diff>
--- a/docs/reports/2026-08-06_功能开发计划_v3.xlsx
+++ b/docs/reports/2026-08-06_功能开发计划_v3.xlsx
@@ -4126,24 +4126,24 @@
           <t>v0.4.5-alpha：admin + UI（list_filter + 批量 action）</t>
         </is>
       </c>
-      <c r="C45" s="52" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D45" s="38" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="E45" s="35" t="inlineStr">
-        <is>
-          <t>待办</t>
-        </is>
-      </c>
-      <c r="F45" s="53" t="inlineStr">
-        <is>
-          <t>DRAFT</t>
+      <c r="C45" s="59" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D45" s="78" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E45" s="63" t="inlineStr">
+        <is>
+          <t>已发布</t>
+        </is>
+      </c>
+      <c r="F45" s="79" t="inlineStr">
+        <is>
+          <t>e4a3707</t>
         </is>
       </c>
       <c r="G45" s="35" t="inlineStr">
@@ -4159,9 +4159,9 @@
       <c r="I45" s="30" t="n">
         <v>0.3</v>
       </c>
-      <c r="J45" s="54" t="inlineStr">
-        <is>
-          <t>admin list_filter 加 task_type；admin action 加 "批量重建"；progress.html 适配 rebuild 无工单场景</t>
+      <c r="J45" s="80" t="inlineStr">
+        <is>
+          <t>admin 加 task_type 筛选+徽章+批量 action；新建 progress_rebuild.html 适配 rebuild 任务</t>
         </is>
       </c>
       <c r="K45" s="32" t="inlineStr">

</xml_diff>

<commit_message>
docs(reports): v0.4.5-alpha queue+归档联动 commit 5 标已发布
</commit_message>
<xml_diff>
--- a/docs/reports/2026-08-06_功能开发计划_v3.xlsx
+++ b/docs/reports/2026-08-06_功能开发计划_v3.xlsx
@@ -4181,24 +4181,24 @@
           <t>v0.4.5-alpha：排队 + 关联归档（services/queue.py）</t>
         </is>
       </c>
-      <c r="C46" s="52" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D46" s="38" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="E46" s="35" t="inlineStr">
-        <is>
-          <t>待办</t>
-        </is>
-      </c>
-      <c r="F46" s="53" t="inlineStr">
-        <is>
-          <t>DRAFT</t>
+      <c r="C46" s="59" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D46" s="78" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E46" s="63" t="inlineStr">
+        <is>
+          <t>已发布</t>
+        </is>
+      </c>
+      <c r="F46" s="79" t="inlineStr">
+        <is>
+          <t>a982d62</t>
         </is>
       </c>
       <c r="G46" s="35" t="inlineStr">
@@ -4214,9 +4214,9 @@
       <c r="I46" s="30" t="n">
         <v>0.5</v>
       </c>
-      <c r="J46" s="54" t="inlineStr">
-        <is>
-          <t>同表冲突排队（FIFO）；归档联动 auto_link_archive opt-in 开关</t>
+      <c r="J46" s="80" t="inlineStr">
+        <is>
+          <t>新建 services/queue.py（同表 FIFO + 归档联动 hook）；rebuild_start 改 409→入队；poller 终态自动推进</t>
         </is>
       </c>
       <c r="K46" s="32" t="inlineStr">

</xml_diff>

<commit_message>
docs(reports): v0.4.5-alpha 134 dev 演练 commit 6 标已发布
</commit_message>
<xml_diff>
--- a/docs/reports/2026-08-06_功能开发计划_v3.xlsx
+++ b/docs/reports/2026-08-06_功能开发计划_v3.xlsx
@@ -4236,24 +4236,24 @@
           <t>v0.4.5-alpha：134 dev 演练（accesscard_black_detail 造碎片 → 重建）</t>
         </is>
       </c>
-      <c r="C47" s="52" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D47" s="38" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="E47" s="35" t="inlineStr">
-        <is>
-          <t>待办</t>
-        </is>
-      </c>
-      <c r="F47" s="53" t="inlineStr">
-        <is>
-          <t>DRAFT</t>
+      <c r="C47" s="59" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="D47" s="78" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E47" s="63" t="inlineStr">
+        <is>
+          <t>已发布</t>
+        </is>
+      </c>
+      <c r="F47" s="79" t="inlineStr">
+        <is>
+          <t>8e40d26</t>
         </is>
       </c>
       <c r="G47" s="35" t="inlineStr">
@@ -4269,9 +4269,9 @@
       <c r="I47" s="30" t="n">
         <v>0.4</v>
       </c>
-      <c r="J47" s="54" t="inlineStr">
-        <is>
-          <t>删 50% 数据造碎片 → 跑 rebuild → 前后对比 INFORMATION_SCHEMA.TABLES.DATA_FREE</t>
+      <c r="J47" s="80" t="inlineStr">
+        <is>
+          <t>134 dev 演练：241558 行 18-21s 重建 + 3 task FIFO 串行 54s；修 5 bug（instance 字段/alter 子句/rebuild_mode/task 字段/is_alive 排队）</t>
         </is>
       </c>
       <c r="K47" s="32" t="inlineStr">

</xml_diff>